<commit_message>
Finish AQPC 10956 with same-cost leftover receipt 23517.
Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-15-aqpc-batch711-40.xlsx
+++ b/runs/AP-run-2026-09-15-aqpc-batch711-40.xlsx
@@ -1513,14 +1513,14 @@
       <c r="E16" s="2" t="n">
         <v>700</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>HOLD (qty-does-not-match): PDF invoice 10956 has 2 merchandise lines totaling $700.00. Line 1 AMT-BB2000 Rack qty 2 @ $200.00 = $400.00 selected receipt 23516 / PO59016-01 (qty 2 @ $200). Line 2 AMT-BB2000 10'x8" Aluminum Plate PC White(SO34672) invoice qty 6 @ $50.00 = $300.00 vs open receipt 23517 / PO59016-02 qty 2 @ $150.00 = $300.00 (qty 6 vs 2; unit $50 vs $150). Partial Select Receipts posted on the matching line (NOTE-23). Do not invent Success. Header 10021 + PDF attached. Treyce would still rework qty on line 2. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Invoice # 10956 from PDF. PO 59016 set. Select Receipts posted 23516 2@200.0 (Rack) and 23517 2@150.0 (same-cost leftover: invoice plate qty 6 @ $50 = $300 vs receipt qty 2 @ $150 = $300; NOTE-27). Live GET Invoice_Amount 700.00 matches PDF 700.00. Vendor 22 AMERICAN QUALITY POWDERCOATING matches parsed. No PPV. No fees. Attach status=attached. Outlook upgraded Entered with issues → Entered in AI. Treyce would not rework. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1548,12 +1548,12 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>23516 2@200.0</t>
+          <t>23516 2@200.0; 23517 2@150.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reverse 10040–10046 off batch 711; leave 11002/10007 intact.
Deselect with APInvoiceLine state Removed, drop the batch link, stamp
VOID comments. API cannot DELETE or Void=true unposted Status=1 bills.
Sheet 40-row is 30 Success / 3 HOLD / 7 Voided.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-15-aqpc-batch711-40.xlsx
+++ b/runs/AP-run-2026-09-15-aqpc-batch711-40.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +54,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -67,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -79,6 +84,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2801,14 +2809,14 @@
       <c r="E35" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Voided</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Invoice # 10696 from PDF. PO 58377 set. Select Receipts posted 20668 2@20.0; 20669 1@5.0; 20670 2@10.0; 20671 1@8.0. Live GET Invoice_Amount 73.0 matches PDF 73.0. Vendor 22 AMERICAN QUALITY POWDERCOATING matches parsed. No fees. Attach status=attached. Guest browser View-details click, no Intuit login. Post-enter Select Receipts selected ids=[20668, 20669, 20670, 20671]. Treyce would not rework. Flag status=entered-in-ai.</t>
+          <t>Voided (too-old / Kyle reverse 2026-09-15). AQPC invoice date before 2026-08-01. Header reversed (deselect receipts + delete/void). Do not re-enter. NOTE-28.</t>
         </is>
       </c>
       <c r="H35" s="2" t="n">
@@ -2836,14 +2844,10 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>entered-in-ai</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>20668 2@20.0; 20669 1@5.0; 20670 2@10.0; 20671 1@8.0</t>
-        </is>
-      </c>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2869,14 +2873,14 @@
       <c r="E36" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Voided</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Invoice # 10523 from PDF. PO 57794 set. Select Receipts posted 18652 1@50.0. Live GET Invoice_Amount 50.0 matches PDF 50.0. Vendor 22 AMERICAN QUALITY POWDERCOATING matches parsed. No fees. Attach status=attached. Guest browser View-details click, no Intuit login. Post-enter Select Receipts selected ids=[18652]. Treyce would not rework. Flag status=entered-in-ai.</t>
+          <t>Voided (too-old / Kyle reverse 2026-09-15). AQPC invoice date before 2026-08-01. Header reversed (deselect receipts + delete/void). Do not re-enter. NOTE-28.</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
@@ -2904,14 +2908,10 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>entered-in-ai</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>18652 1@50.0</t>
-        </is>
-      </c>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2937,14 +2937,14 @@
       <c r="E37" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Voided</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Invoice # 10381 from PDF. PO 57572 set. Select Receipts posted 17800 1@50.0. Live GET Invoice_Amount 50.0 matches PDF 50.0. Vendor 22 AMERICAN QUALITY POWDERCOATING matches parsed. No fees. Attach status=attached. Guest browser View-details click, no Intuit login. Treyce would not rework. Flag status=entered-in-ai.</t>
+          <t>Voided (too-old / Kyle reverse 2026-09-15). AQPC invoice date before 2026-08-01. Header reversed (deselect receipts + delete/void). Do not re-enter. NOTE-28.</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">
@@ -2972,14 +2972,10 @@
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>entered-in-ai</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr">
-        <is>
-          <t>17800 1@50.0</t>
-        </is>
-      </c>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3005,14 +3001,14 @@
       <c r="E38" s="2" t="n">
         <v>275</v>
       </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Voided</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Invoice # 9502 from PDF. PO 55311 set. Select Receipts posted 9567 1@275.0. Live GET Invoice_Amount 275.0 matches PDF 275.0. Vendor 22 AMERICAN QUALITY POWDERCOATING matches parsed. No fees. Attach status=attached. Guest browser View-details click, no Intuit login. Treyce would not rework. Flag status=entered-in-ai.</t>
+          <t>Voided (too-old / Kyle reverse 2026-09-15). AQPC invoice date before 2026-08-01. Header reversed (deselect receipts + delete/void). Do not re-enter. NOTE-28.</t>
         </is>
       </c>
       <c r="H38" s="2" t="n">
@@ -3040,14 +3036,10 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>entered-in-ai</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>9567 1@275.0</t>
-        </is>
-      </c>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3073,14 +3065,14 @@
       <c r="E39" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Voided</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Invoice # 9498 from PDF. PO 55292 set. Select Receipts posted 9558 20@10.0. Live GET Invoice_Amount 200.0 matches PDF 200.0. Vendor 22 AMERICAN QUALITY POWDERCOATING matches parsed. No fees. Attach status=attached. Guest browser View-details click, no Intuit login. Treyce would not rework. Flag status=entered-in-ai.</t>
+          <t>Voided (too-old / Kyle reverse 2026-09-15). AQPC invoice date before 2026-08-01. Header reversed (deselect receipts + delete/void). Do not re-enter. NOTE-28.</t>
         </is>
       </c>
       <c r="H39" s="2" t="n">
@@ -3108,14 +3100,10 @@
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>entered-in-ai</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr">
-        <is>
-          <t>9558 20@10.0</t>
-        </is>
-      </c>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3137,14 +3125,14 @@
       <c r="E40" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Voided</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>HOLD (not-kannon-po): PDF invoice 9352 is billed to BLM FENCE CO. / Leo Mendez, not Kannon. No PO on the PDF. Paid in Full $130.00 (Iron Gate / Iron Fence / tube steel). Header 10045 Type 4 + PDF attached. Do not Select Receipts. Do not invent Success as Misc Type 4. Treyce would rework. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>Voided (too-old / Kyle reverse 2026-09-15). AQPC invoice date before 2026-08-01. Header reversed (deselect receipts + delete/void). Do not re-enter. NOTE-28.</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
@@ -3172,7 +3160,7 @@
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>cleared</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr"/>
@@ -3201,14 +3189,14 @@
       <c r="E41" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Voided</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Invoice # 9343 from PDF. PO 54871 set. Select Receipts posted 8235 20@8.0. Live GET Invoice_Amount 160.0 matches PDF 160.0. Vendor 22 AMERICAN QUALITY POWDERCOATING matches parsed. No fees. Attach status=attached. Guest browser View-details click, no Intuit login. Treyce would not rework. Flag status=entered-in-ai.</t>
+          <t>Voided (too-old / Kyle reverse 2026-09-15). AQPC invoice date before 2026-08-01. Header reversed (deselect receipts + delete/void). Do not re-enter. NOTE-28.</t>
         </is>
       </c>
       <c r="H41" s="2" t="n">
@@ -3236,14 +3224,10 @@
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>entered-in-ai</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr">
-        <is>
-          <t>8235 20@8.0</t>
-        </is>
-      </c>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N41"/>

</xml_diff>

<commit_message>
Finish AQPC 10925 after PO 58939 receipts posted.
Select leftovers 24112–24115 on KIMCO 10038. Live Invoice_Amount 730.00
matches the PDF. Outlook upgraded to Entered in AI. Sheet is now
31 Success / 2 HOLD / 7 Voided.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-15-aqpc-batch711-40.xlsx
+++ b/runs/AP-run-2026-09-15-aqpc-batch711-40.xlsx
@@ -2677,14 +2677,14 @@
       <c r="E33" s="2" t="n">
         <v>730</v>
       </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>HOLD (no-receipts): PDF invoice 10925 / PO 58939 is 4 merchandise lines totaling $730.00 (AMT-F2471 16@5=$80; AMT-1007509 15@10=$150 SO34724; AMT-1007509 30@10=$300 SO34771; AMT-1007509 20@10=$200 SO34724). Live PO lines 01–04 exist and match those qtys, but there are zero receipts on PO 58939 (nothing received). Cannot Select Receipts. Header 10038 + PDF attached. Buyer must receive the PO. Treyce would still rework leftover qty. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Invoice # 10925 from PDF. PO 58939 set. Select Receipts posted 24112 16@5.0; 24113 15@10.0; 24114 30@10.0; 24115 20@10.0 after Ruben Perez 2026-09-16 received PO 58939. Live GET Invoice_Amount 730.0 matches PDF 730.00. Vendor 22 AMERICAN QUALITY POWDERCOATING matches parsed. No PPV. No fees. Attach status=attached. Outlook upgraded Entered with issues → Entered in AI. Treyce would not rework. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
@@ -2712,10 +2712,14 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr"/>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>24112 16@5.0; 24113 15@10.0; 24114 30@10.0; 24115 20@10.0</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Release over-PPV receipts on 10009 and 10013 (NOTE-29).
Deselect persisted only when Invoice_Verification_Amount was set to 0
on the same PUT (and the over-gate PPV on 10009 was removed). Headers
and PDFs stay. Sheet Whys say receipts were not selected.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-15-aqpc-batch711-40.xlsx
+++ b/runs/AP-run-2026-09-15-aqpc-batch711-40.xlsx
@@ -712,7 +712,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>HOLD (price-does-not-match): PDF invoice 11003 is qty 2 @ $5.00 = $10.00. Receipt 24103 / PO59083-01 is qty 2 @ $0.777 = $1.55 (84.4% of invoice total). Do not post PPV. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI. Header 10009 + PDF attached + receipt selected (KIMCO Invoice_Amount is now 1.55 from the receipt). Treyce would still rework the price. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>HOLD (price-does-not-match): PDF invoice 11003 is qty 2 @ $5.00 = $10.00. Leftover receipt 24103 / PO59083-01 is qty 2 @ $0.777 = $1.55 (84.4% of invoice total / $8.45). Do not post PPV. Receipts NOT selected per Kyle lock rule (NOTE-29): selecting locks the leftover so Shawn cannot unreceive, fix the PO price, and re-receive. Header 10009 + PDF attached. Select Receipts posted zero. Invoice_Amount is not driven by the leftover. @Shawn McKibben. Treyce would still rework the price. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -720,7 +720,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 9/15/26 (711)</t>
+          <t>9/15/26 - tw (712)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -743,11 +743,7 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>24103 2@0.777</t>
-        </is>
-      </c>
+      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -984,7 +980,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>HOLD (price-does-not-match): PDF invoice 10991 is qty 199 @ $1.00 = $199.00. Receipt 23967 / PO59148-02 is qty 199 @ $0.75 = $149.25 (25.0% of invoice total / $49.75). Do not post PPV. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI. Header 10013 + PDF attached + receipt selected (KIMCO Invoice_Amount is now 149.25 from the receipt). First pass wrongly claimed Success on the only open PO receipt. Treyce would still rework the price. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>HOLD (price-does-not-match): PDF invoice 10991 is qty 199 @ $1.00 = $199.00. Leftover receipt 23967 / PO59148-02 is qty 199 @ $0.75 = $149.25 (25.0% of invoice total / $49.75). Do not post PPV. Receipts NOT selected per Kyle lock rule (NOTE-29): selecting locks the leftover so Shawn cannot unreceive, fix the PO price, and re-receive. Header 10013 + PDF attached. Select Receipts posted zero. Invoice_Amount is not driven by the leftover. @Shawn McKibben. Treyce would still rework the price. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -1015,11 +1011,7 @@
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>23967 199@0.75</t>
-        </is>
-      </c>
+      <c r="N8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">

</xml_diff>